<commit_message>
feat: implement tests for TC 08-15
</commit_message>
<xml_diff>
--- a/assets/test-cases/TestCases_1.0.xlsx
+++ b/assets/test-cases/TestCases_1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\LEARNING\QA Engineer\Internship\9t-cypres-cucumber-telnyx\assets\test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D17E51A-E99D-408E-9789-C44834D1D09A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D12C6D-7FA7-4F1A-9D7D-D652735D6DED}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -392,9 +392,6 @@
     <t>Verify estimated cost is updated based on the entered monthly volume</t>
   </si>
   <si>
-    <t>Verify the Report Abuse form displays validation after submission an empty form</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">The </t>
     </r>
@@ -419,308 +416,6 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> page is opened</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Scroll to </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> section
-2. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> link
-3. Scroll to </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Submit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-4. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Submit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button
-5. Verify several "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>This field is required</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>" messages are displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> section was displayed
-2. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> page was opened
-3. The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Submit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button was displayed
-4. The page was scrolled to the top
-5. The several "</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>This field is required</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>" messages were displayed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">The </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> page is opened</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. Fill all mandatory fields with valid data
-2. Click the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Submit</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> button</t>
-    </r>
-  </si>
-  <si>
-    <t>Verify the Report Abuse form can be submitted with valid data"</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. The mandatory fields were populated with valid data
-2. A confirmation message is displayed on the </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Report Abuse</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> page</t>
     </r>
   </si>
   <si>
@@ -3171,6 +2866,378 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> options were displayed in search results</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> header button
+2. Verify the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Voice API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> category is visible
+3. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Voice API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> category
+4. Scroll to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Download SIP Trunking Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> form
+5. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Submit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify the Download SIP Trunking Pricing form displays validation messages after empty submission</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mega menu was displayed
+2. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Voice API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> category was visible
+3. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Voice API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> page was opened
+4. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Download SIP Trunking Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> form was displayed
+5. The "</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>This field is required</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>" message was displayed</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify the Download SIP Trunking Pricing form can be submitted using valid data</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Voice API</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> page is opened</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. Scroll to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Download SIP Trunking Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> form
+2. Fill all mandatory fields with valid data
+3. Click the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Submit</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> button</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. The </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Download SIP Trunking Pricing</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> form was displayed
+2. The mandatory fields were populated with valid data
+3. A confirmation message was displayed on the </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>new</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> page</t>
     </r>
   </si>
 </sst>
@@ -3578,10 +3645,10 @@
         <v>14</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>7</v>
@@ -3598,10 +3665,10 @@
         <v>16</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
@@ -3618,10 +3685,10 @@
         <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>7</v>
@@ -3638,10 +3705,10 @@
         <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>8</v>
@@ -3658,10 +3725,10 @@
         <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>7</v>
@@ -3692,16 +3759,16 @@
         <v>20</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>7</v>
@@ -3718,10 +3785,10 @@
         <v>16</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>7</v>
@@ -3732,36 +3799,36 @@
         <v>22</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>35</v>
+        <v>69</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>38</v>
+        <v>70</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>71</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>40</v>
+        <v>73</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>42</v>
+        <v>74</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>6</v>
@@ -3772,16 +3839,16 @@
         <v>24</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>7</v>
@@ -3792,16 +3859,16 @@
         <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>6</v>
@@ -3812,16 +3879,16 @@
         <v>26</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>7</v>
@@ -3832,16 +3899,16 @@
         <v>27</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>7</v>
@@ -3852,16 +3919,16 @@
         <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>6</v>

</xml_diff>